<commit_message>
fix: populate Excel EC2 Memory Utilization column from memory_avg_display
The EC2 sheet read memory via inst.get('memory_max'), but mock/reference
data now supplies memory_avg_display, leaving the Memory Utilization column
blank. Add ReportStyles.memory_cell (mirrors the Word report helper:
prefer memory_avg_display, fall back to numeric memory_avg/memory_max) and
use it in ec2_sheet so Excel matches the Word report. Numeric values stay
floats so conditional formatting still applies; '-' rows stay '-'.
Regenerate demo docx/xlsx (14-20 Sep 2026, mock).
</commit_message>
<xml_diff>
--- a/demo/Fly91_Weekly_AWS_BAU_Report_14-20_Sep_2026.xlsx
+++ b/demo/Fly91_Weekly_AWS_BAU_Report_14-20_Sep_2026.xlsx
@@ -2237,7 +2237,7 @@
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>October 05, 2026  12:16 AM</t>
+          <t>October 05, 2026  06:56 PM</t>
         </is>
       </c>
     </row>
@@ -4667,10 +4667,8 @@
       <c r="F6" s="25" t="n">
         <v>9.19</v>
       </c>
-      <c r="G6" s="25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G6" s="25" t="n">
+        <v>50.62</v>
       </c>
       <c r="H6" s="25" t="inlineStr">
         <is>
@@ -4703,10 +4701,8 @@
       <c r="F7" s="24" t="n">
         <v>8.869999999999999</v>
       </c>
-      <c r="G7" s="24" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G7" s="24" t="n">
+        <v>48.23</v>
       </c>
       <c r="H7" s="24" t="inlineStr">
         <is>
@@ -4739,10 +4735,8 @@
       <c r="F8" s="25" t="n">
         <v>3.89</v>
       </c>
-      <c r="G8" s="25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G8" s="25" t="n">
+        <v>25.35</v>
       </c>
       <c r="H8" s="25" t="inlineStr">
         <is>
@@ -4775,10 +4769,8 @@
       <c r="F9" s="24" t="n">
         <v>1.8</v>
       </c>
-      <c r="G9" s="24" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G9" s="24" t="n">
+        <v>73.97</v>
       </c>
       <c r="H9" s="24" t="inlineStr">
         <is>
@@ -4853,10 +4845,8 @@
       <c r="F11" s="24" t="n">
         <v>14.3</v>
       </c>
-      <c r="G11" s="24" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G11" s="24" t="n">
+        <v>55.21</v>
       </c>
       <c r="H11" s="24" t="inlineStr">
         <is>
@@ -4889,10 +4879,8 @@
       <c r="F12" s="25" t="n">
         <v>5.77</v>
       </c>
-      <c r="G12" s="25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G12" s="25" t="n">
+        <v>48.75</v>
       </c>
       <c r="H12" s="25" t="inlineStr">
         <is>
@@ -4925,10 +4913,8 @@
       <c r="F13" s="24" t="n">
         <v>5.15</v>
       </c>
-      <c r="G13" s="24" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G13" s="24" t="n">
+        <v>9.220000000000001</v>
       </c>
       <c r="H13" s="24" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix: populate Excel RDS sheet from display-string fields (mock parity with Word)
</commit_message>
<xml_diff>
--- a/demo/Fly91_Weekly_AWS_BAU_Report_14-20_Sep_2026.xlsx
+++ b/demo/Fly91_Weekly_AWS_BAU_Report_14-20_Sep_2026.xlsx
@@ -2237,7 +2237,7 @@
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>October 05, 2026  06:56 PM</t>
+          <t>October 05, 2026  07:00 PM</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2335,7 @@
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>fly91-data-science-production-db</t>
         </is>
       </c>
       <c r="B4" s="24" t="inlineStr">
@@ -2345,39 +2345,39 @@
       </c>
       <c r="C4" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>db.t4g.small</t>
         </is>
       </c>
       <c r="D4" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3.78%</t>
         </is>
       </c>
       <c r="E4" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>30.61%</t>
         </is>
       </c>
       <c r="F4" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>8.74%</t>
         </is>
       </c>
       <c r="G4" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0.5 GB out of 2GB</t>
         </is>
       </c>
       <c r="H4" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>15.8GB out of 20 GB</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>fly91-db</t>
         </is>
       </c>
       <c r="B5" s="25" t="inlineStr">
@@ -2387,39 +2387,39 @@
       </c>
       <c r="C5" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>db.r7g.large</t>
         </is>
       </c>
       <c r="D5" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2.9%</t>
         </is>
       </c>
       <c r="E5" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>47.49%</t>
         </is>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3.72%</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.86GB out of 16 GB</t>
         </is>
       </c>
       <c r="H5" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>89.1GB out of 100 GB</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>fly91-dev-db</t>
         </is>
       </c>
       <c r="B6" s="24" t="inlineStr">
@@ -2429,39 +2429,39 @@
       </c>
       <c r="C6" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>db.t3.large</t>
         </is>
       </c>
       <c r="D6" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14.41%</t>
         </is>
       </c>
       <c r="E6" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="F6" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>46.17%</t>
         </is>
       </c>
       <c r="G6" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0.86GB out of 8 GB</t>
         </is>
       </c>
       <c r="H6" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>21.4GB out of 30 GB</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>fly91-development-psql</t>
         </is>
       </c>
       <c r="B7" s="25" t="inlineStr">
@@ -2471,39 +2471,39 @@
       </c>
       <c r="C7" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>db.t3.medium</t>
         </is>
       </c>
       <c r="D7" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4.44%</t>
         </is>
       </c>
       <c r="E7" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>79.77%</t>
         </is>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13.32%</t>
         </is>
       </c>
       <c r="G7" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2.90GB out of 4 GB</t>
         </is>
       </c>
       <c r="H7" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0.8GB out of 77 GB</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>fly91-prod-psql-db</t>
         </is>
       </c>
       <c r="B8" s="24" t="inlineStr">
@@ -2513,39 +2513,39 @@
       </c>
       <c r="C8" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>db.t3.large</t>
         </is>
       </c>
       <c r="D8" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>5.92%</t>
         </is>
       </c>
       <c r="E8" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="F8" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>43.76%</t>
         </is>
       </c>
       <c r="G8" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4.35GB out of 8 GB</t>
         </is>
       </c>
       <c r="H8" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>9.0GB out of 100 GB</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>fly91-uat-psql-db</t>
         </is>
       </c>
       <c r="B9" s="25" t="inlineStr">
@@ -2555,32 +2555,32 @@
       </c>
       <c r="C9" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>db.t3.medium</t>
         </is>
       </c>
       <c r="D9" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>5.65%</t>
         </is>
       </c>
       <c r="E9" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>99.57%</t>
         </is>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>39.4%</t>
         </is>
       </c>
       <c r="G9" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2.00GB out of 4 GB</t>
         </is>
       </c>
       <c r="H9" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>27.1GB out of 50 GB</t>
         </is>
       </c>
     </row>
@@ -2616,132 +2616,132 @@
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>fly91-data-science-production-db</t>
         </is>
       </c>
       <c r="B16" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>817.54 KB</t>
         </is>
       </c>
       <c r="C16" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>77.25 KB</t>
         </is>
       </c>
       <c r="D16" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>5</t>
         </is>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>fly91-db</t>
         </is>
       </c>
       <c r="B17" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>24.70 MB</t>
         </is>
       </c>
       <c r="C17" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>9.52 MB</t>
         </is>
       </c>
       <c r="D17" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12</t>
         </is>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>fly91-dev-db</t>
         </is>
       </c>
       <c r="B18" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>15.78 MB</t>
         </is>
       </c>
       <c r="C18" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>142.12 KB</t>
         </is>
       </c>
       <c r="D18" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>68</t>
         </is>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>fly91-development-psql</t>
         </is>
       </c>
       <c r="B19" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>15.58 MB</t>
         </is>
       </c>
       <c r="C19" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2.50 MB</t>
         </is>
       </c>
       <c r="D19" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>134</t>
         </is>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>fly91-prod-psql-db</t>
         </is>
       </c>
       <c r="B20" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>9.79 MB</t>
         </is>
       </c>
       <c r="C20" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2.21 MB</t>
         </is>
       </c>
       <c r="D20" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>210</t>
         </is>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>fly91-uat-psql-db</t>
         </is>
       </c>
       <c r="B21" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18.92 MB</t>
         </is>
       </c>
       <c r="C21" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>772.02 KB</t>
         </is>
       </c>
       <c r="D21" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>193</t>
         </is>
       </c>
     </row>

</xml_diff>